<commit_message>
SPM-53: Notify equipment changes and fulfilment outcomes
Technical Support are told when the coordinator adds, removes or changes
the quantity of an equipment requirement (AC10); the coordinator when a
line is Reserved, Partially fulfilled or Cannot be provided (AC11). As an
important change, each equipment change also tells the organiser, and
says when it moved a Confirmed event back to Planning (AC14, AC15).
SPM-53-TC10 checks the organiser's notifications too.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-53_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-53_Test_Cases.xlsx
@@ -912,12 +912,12 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Technical Support are notified when the coordinator adds, changes the quantity of and removes equipment on a Planning event</t>
+          <t>Technical Support, and the organiser, are notified when the coordinator adds, changes the quantity of and removes equipment on a Planning event</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>AC10</t>
+          <t>AC10, AC14</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -1663,7 +1663,8 @@
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>SPM-53-TC13
+          <t>SPM-53-TC10
+SPM-53-TC13
 SPM-53-TC14
 SPM-53-TC15
 SPM-53-TC16</t>
@@ -2288,7 +2289,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Technical Support are notified when the coordinator adds, changes the quantity of and removes equipment on a Planning event</t>
+          <t>Technical Support, and the organiser, are notified when the coordinator adds, changes the quantity of and removes equipment on a Planning event</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2306,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="206.5" customHeight="1">
+    <row r="5" ht="247" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2322,7 +2323,9 @@
 7. Log out and log in as Technical Support Kenji Sato (kenji.sato@connectsphere.com / password123)
 8. Click 'Notifications' in the sidebar
 9. Log out and log in as Technical Support Aisha Omar (aisha.omar@connectsphere.com / password123)
-10. Click 'Notifications' in the sidebar</t>
+10. Click 'Notifications' in the sidebar
+11. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+12. Click 'Notifications' in the sidebar</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2344,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="166" customHeight="1">
+    <row r="7" ht="220" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2353,7 +2356,8 @@
 Step 4: The 'Save' button disappears and the row shows Quantity 3.
 Step 6: The 'SPM53 Lectern Mic' row disappears.
 Step 8: Three unread notifications 'Equipment requirement changed' for 'SPM53 Harbour Equipment Fair' are listed, newest first, with the messages 'SPM53 Lectern Mic was removed from "SPM53 Harbour Equipment Fair".', 'SPM53 Projector on "SPM53 Harbour Equipment Fair" changed from 2 to 3.' and 'SPM53 Speaker × 1 was added to "SPM53 Harbour Equipment Fair".'
-Step 10: Aisha Omar's list has the same three notifications.</t>
+Step 10: Aisha Omar's list has the same three notifications.
+Step 12: Three unread notifications 'Event information changed' for 'SPM53 Harbour Equipment Fair' are listed, each with the message '"SPM53 Harbour Equipment Fair" has changed: Equipment requirements.'</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2876,7 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 before and after this case (it decides a change request). 'SPM53 Harbour Change Review' (Planning, 30 people) has a pending change request from Rachel Ng for three fields: Event name, Expected attendance and Description.
+          <t>Run npm run fixtures:spm53 before and after this case (it decides a change request). 'SPM53 Harbour Change Review' (Planning, 30 people) has a pending change request from Rachel Ng for three fields: Event name, Description and Expected attendance.
 Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
         </is>
       </c>
@@ -2888,7 +2892,7 @@
           <t>1. Click 'Change Requests' in the sidebar
 2. Click 'Review' on the request for 'SPM53 Harbour Change Review'
 3. For 'Event name', choose 'Reject' and enter the reason
-4. For 'Expected attendance' and 'Description', choose 'Approve'
+4. For 'Description' and 'Expected attendance', choose 'Approve'
 5. Click 'Save decision'
 6. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
 7. Click 'Notifications' in the sidebar</t>
@@ -2919,7 +2923,7 @@
       <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 5: 'Change request processed.' is shown and the request is Partially approved.
-Step 7: Two unread notifications for 'SPM53 Harbour Change Review' are listed: 'Change request partially approved' with the message 'Your change request for "SPM53 Harbour Change Review" was partially approved. Event name: rejected – The invitations have already gone out. Expected attendance: approved. Description: approved.', and 'Event information changed' with the message '"SPM53 Harbour Change Review" has changed: Expected attendance.'</t>
+Step 7: Two unread notifications for 'SPM53 Harbour Change Review' are listed: 'Change request partially approved' with the message 'Your change request for "SPM53 Harbour Change Review" was partially approved. Event name: rejected – The invitations have already gone out. Description: approved. Expected attendance: approved.', and 'Event information changed' with the message '"SPM53 Harbour Change Review" has changed: Expected attendance.'</t>
         </is>
       </c>
     </row>
@@ -3763,7 +3767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3821,24 +3825,24 @@
       </c>
       <c r="C4" s="11" t="n"/>
     </row>
-    <row r="5" ht="58" customHeight="1">
+    <row r="5" ht="98.5" customHeight="1">
       <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-29: AC17 'rescheduled' is any change to the event's date or time, whether the coordinator saves it (SPM-62) or it is applied from an approved change request (SPM-32, including a Postponed event given its new date).</t>
+          <t>DECIDED 2026-10-29: Equipment is one of AC14's important changes, and SPM-62 already treats every saved change to an equipment requirement (including its technical requirements) as one, moving a Confirmed event back to Planning. So each such save tells the organiser 'Event information changed' naming 'Equipment requirements', and 'Event no longer confirmed' when it moved a Confirmed event back (AC15). Technical Support hear only of adds, removals and quantity changes (AC10).</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
     </row>
-    <row r="6" ht="44.5" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-29: AC16 'registered' includes an attendee who accepts a waiting-list offer (SPM-66), since that registers them. Joining the waiting list is not registering and notifies nobody.</t>
+          <t>DECIDED 2026-10-29: AC17 'rescheduled' is any change to the event's date or time, whether the coordinator saves it (SPM-62) or it is applied from an approved change request (SPM-32, including a Postponed event given its new date).</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
@@ -3849,18 +3853,18 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-29: AC18 Completed includes an event the 7-day sweep completes (SPM-36 AC6). It has no manual case, since the sweep acts on an event 7 days after it ends; the unit tests cover it.</t>
+          <t>DECIDED 2026-10-29: AC16 'registered' includes an attendee who accepts a waiting-list offer (SPM-66), since that registers them. Joining the waiting list is not registering and notifies nobody.</t>
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
     </row>
-    <row r="8" ht="58" customHeight="1">
+    <row r="8" ht="44.5" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-29: AC15's second route, a safety check closed after a change (SPM-88), moves an event from Safety review or Safety approved to Planning, never from Confirmed, so only an important change to a Confirmed event (SPM-62) raises 'Event no longer confirmed'.</t>
+          <t>DECIDED 2026-10-29: AC18 Completed includes an event the 7-day sweep completes (SPM-36 AC6). It has no manual case, since the sweep acts on an event 7 days after it ends; the unit tests cover it.</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>
@@ -3871,10 +3875,21 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
+          <t>DECIDED 2026-10-29: AC15's second route, a safety check closed after a change (SPM-88), moves an event from Safety review or Safety approved to Planning, never from Confirmed, so only an important change to a Confirmed event (SPM-62) raises 'Event no longer confirmed'.</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
           <t>OPEN 2026-10-29: AC16's 'including when the Event Coordinator adds them (SPM-57)' cannot be built or tested until SPM-57 (Manually Add Attendee, PR #92) is merged. Whoever merges second adds the notification to the coordinator's add, using the 'Registration confirmed' wording.</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
SPM-53: One test case per acceptance criterion
21 short cases, at least one for each of the 20 criteria. A case that
follows on the same event continues from the one before it instead of
repeating its setup. Adds the two fixture events the AC14 and AC19/AC20
cases need.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-53_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-53_Test_Cases.xlsx
@@ -14,6 +14,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC05" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC06" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC07" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC12" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC13" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC14" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC15" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC16" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC17" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC18" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC19" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC20" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC21" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -453,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -546,12 +560,12 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Submitting a request notifies every Event Coordinator Lead, and assigning then reassigning it notifies each coordinator and the organiser</t>
+          <t>Submitting an event request notifies every active Event Coordinator Lead, naming the event</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC5, AC6, AC7, AC19, AC20</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -585,12 +599,12 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>The organiser hears of a clarification request and of the approval or rejection, the coordinator hears it was answered, and nobody else is told the outcome</t>
+          <t>Assigning a coordinator tells the organiser the coordinator's name</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>AC2, AC3, AC4</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
@@ -624,12 +638,12 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>A venue booking request notifies every Venue Staff user, and the coordinator hears each approval and rejection with the venue, times and reason</t>
+          <t>The newly assigned coordinator is notified of the assignment</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>AC8, AC9</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -663,12 +677,12 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Equipment added, changed and removed notifies Technical Support and the organiser, and each fulfilment outcome notifies the coordinator</t>
+          <t>Reassigning notifies the new coordinator and the organiser, and tells the previous coordinator the event is no longer theirs</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>AC10, AC11, AC14</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -702,12 +716,12 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>A change request notifies the coordinator, and a partly approved decision tells the organiser each field's outcome and that the expected attendance changed</t>
+          <t>The organiser is notified when the assigned coordinator asks for clarification, with the message</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>AC12, AC13, AC14</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -741,12 +755,12 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>An ordinary edit notifies nobody; rescheduling a Confirmed event tells the organiser it changed and is no longer confirmed, and tells only Registered attendees the new date</t>
+          <t>The assigned coordinator is notified when the organiser answers the clarification by resubmitting</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>AC14, AC15, AC17</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -780,12 +794,12 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Registering notifies the attendee; confirming, completing, postponing and cancelling notify the organiser, and postponing and cancelling notify only Registered attendees, with any reason</t>
+          <t>An approval and a rejection notify only the organiser, the rejection with its reason</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>AC16, AC18</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
@@ -806,304 +820,568 @@
       <c r="H10" s="11" t="n"/>
       <c r="I10" s="11" t="n"/>
     </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>TC08</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC08</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Sending a venue booking request notifies every active Venue Staff user</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>AC8</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>TC09</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC09</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>The assigned coordinator is notified of a booking approval and a rejection, with the venue, times and reason</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>AC9</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="n"/>
+      <c r="I12" s="11" t="n"/>
+    </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>TC10</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC10</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Technical Support are notified when the coordinator adds, changes the quantity of and removes equipment</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>AC10</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC11</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC11</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>The coordinator is notified when Technical Support mark lines Reserved, Partially fulfilled and Cannot be provided</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>AC11</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="n"/>
+      <c r="I14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>TC12</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC12</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>The assigned coordinator is notified when the organiser sends a change request</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>AC12</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>TC13</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC13</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>A partly approved change request tells the organiser the outcome of each field</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>AC13</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="n"/>
+      <c r="I16" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>TC14</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC14</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>An ordinary edit notifies nobody, and an important change tells the organiser which information changed</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>AC14</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="n"/>
+      <c r="I17" s="11" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>TC15</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC15</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Rescheduling a Confirmed event tells the organiser it changed and is no longer confirmed</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>AC15</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="n"/>
+      <c r="I18" s="11" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>TC16</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC16</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Only attendees whose registration is Registered are told the new date and time</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>AC17</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="n"/>
+      <c r="I19" s="11" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>TC17</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC17</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>An attendee who registers for an event is notified that they are registered</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>AC16</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="n"/>
+      <c r="I20" s="11" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>TC18</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC18</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>The organiser is notified when the coordinator confirms an event and marks one completed</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>AC18</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H21" s="11" t="n"/>
+      <c r="I21" s="11" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>TC19</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC19</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Postponing and cancelling notify the organiser and only the Registered attendees, with the reason when there is one</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>AC18, AC16</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H22" s="11" t="n"/>
+      <c r="I22" s="11" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>TC20</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC20</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>A notification appears in the recipient's list, unread, as soon as it is raised</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>AC19</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="n"/>
+      <c r="I23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>TC21</t>
+        </is>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC21</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Selecting a notification opens the event it is about</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>AC20</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="n"/>
+      <c r="I24" s="11" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="n"/>
-    </row>
-    <row r="14" ht="44.5" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Given an Event Organiser submits an event request, when it is submitted, then every active Event Coordinator Lead is notified, naming the event.</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC01</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="n"/>
-    </row>
-    <row r="15" ht="44.5" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>AC2</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>The Event Organiser who owns the event is notified when the assigned Event Coordinator requests clarification, with the clarification message.</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC02</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="n"/>
-    </row>
-    <row r="16" ht="31" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
-        <is>
-          <t>AC3</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>The assigned Event Coordinator is notified when the Event Organiser responds to an open clarification request.</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC02</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n"/>
-    </row>
-    <row r="17" ht="44.5" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>AC4</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>The Event Organiser who owns the event is notified when the assigned Event Coordinator approves or rejects it, with the reason for a rejection. No other user is notified of the outcome.</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC02</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="n"/>
-    </row>
-    <row r="18" ht="31" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>AC5</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>The Event Organiser who owns the event is notified when an Event Coordinator is assigned, with the Coordinator's name.</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC01</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="17.5" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>AC6</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>The newly assigned Coordinator is notified of the assignment.</t>
-        </is>
-      </c>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC01</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="n"/>
-    </row>
-    <row r="20" ht="58" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>AC7</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>Given an event is reassigned to a different Coordinator, when the reassignment is saved, then the newly assigned Coordinator and the Event Organiser are notified as for an assignment, and the previously assigned Coordinator is notified that the event is no longer theirs.</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC01</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="31" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>AC8</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Every active Venue Staff user is notified when a venue booking request is submitted for review.</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC03</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="44.5" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>AC9</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>The assigned Event Coordinator is notified when Venue Staff approve or reject a venue booking request for the event, with the venue, the requested times and, for a rejection, the reason.</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC03</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="23" ht="58" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>AC10</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Every active Technical Support Staff user is notified when the assigned Event Coordinator adds, removes or changes the quantity of an equipment requirement on an event in Planning or Confirmed (the events listed in the Equipment Requests queue, SPM-48).</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC04</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="n"/>
-    </row>
-    <row r="24" ht="44.5" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>AC11</t>
-        </is>
-      </c>
-      <c r="B24" s="11" t="inlineStr">
-        <is>
-          <t>The assigned Event Coordinator is notified when Technical Support Staff mark an equipment requirement Reserved, Partially fulfilled or Cannot be provided.</t>
-        </is>
-      </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC04</t>
-        </is>
-      </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="25" ht="31" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>AC12</t>
-        </is>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>The assigned Event Coordinator is notified when the Event Organiser submits a change request.</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC05</t>
-        </is>
-      </c>
-      <c r="F25" s="9" t="n"/>
-    </row>
-    <row r="26" ht="31" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>AC13</t>
-        </is>
-      </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>The Event Organiser is notified of the outcome of a change request, including the outcome for each field where it is partially approved.</t>
-        </is>
-      </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC05</t>
-        </is>
-      </c>
-      <c r="F26" s="9" t="n"/>
-    </row>
-    <row r="27" ht="71.5" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>AC14</t>
-        </is>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>Given an important change (date and time, expected attendance, venue requirements or equipment) is saved by the assigned Coordinator or applied from an approved change request, when it is saved, then the Event Organiser who owns the event is notified, naming which of these changed. No other user is notified of the change by this criterion.</t>
         </is>
       </c>
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="9" t="n"/>
-      <c r="E27" s="11" t="inlineStr">
-        <is>
-          <t>SPM-53-TC04
-SPM-53-TC05
-SPM-53-TC06</t>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
         </is>
       </c>
       <c r="F27" s="9" t="n"/>
@@ -1111,39 +1389,39 @@
     <row r="28" ht="44.5" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>AC15</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>The Event Organiser who owns the event is notified when the event moves from Confirmed back to Planning (an important change, SPM-62, or a safety check closed after a change, SPM-88).</t>
+          <t>Given an Event Organiser submits an event request, when it is submitted, then every active Event Coordinator Lead is notified, naming the event.</t>
         </is>
       </c>
       <c r="C28" s="8" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>SPM-53-TC06</t>
+          <t>SPM-53-TC01</t>
         </is>
       </c>
       <c r="F28" s="9" t="n"/>
     </row>
-    <row r="29" ht="58" customHeight="1">
+    <row r="29" ht="44.5" customHeight="1">
       <c r="A29" s="11" t="inlineStr">
         <is>
-          <t>AC16</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>An Attendee is notified when they are registered for an event, including when the Event Coordinator adds them (SPM-57), and when an event they are registered for is Postponed or Cancelled (see the confirmed, completed, postponed or cancelled criterion below).</t>
+          <t>The Event Organiser who owns the event is notified when the assigned Event Coordinator requests clarification, with the clarification message.</t>
         </is>
       </c>
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>SPM-53-TC07</t>
+          <t>SPM-53-TC05</t>
         </is>
       </c>
       <c r="F29" s="9" t="n"/>
@@ -1151,12 +1429,12 @@
     <row r="30" ht="31" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>AC17</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Attendees whose registration is Registered are notified of the new date and time when an event is rescheduled.</t>
+          <t>The assigned Event Coordinator is notified when the Event Organiser responds to an open clarification request.</t>
         </is>
       </c>
       <c r="C30" s="8" t="n"/>
@@ -1168,15 +1446,15 @@
       </c>
       <c r="F30" s="9" t="n"/>
     </row>
-    <row r="31" ht="58" customHeight="1">
+    <row r="31" ht="44.5" customHeight="1">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>AC18</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>The Event Organiser who owns the event is notified when it is Confirmed, Completed, Postponed or Cancelled. Attendees whose registration is Registered are notified when it is Postponed or Cancelled. For Postponed and Cancelled, the notification includes the recorded reason.</t>
+          <t>The Event Organiser who owns the event is notified when the assigned Event Coordinator approves or rejects it, with the reason for a rejection. No other user is notified of the outcome.</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>
@@ -1188,22 +1466,22 @@
       </c>
       <c r="F31" s="9" t="n"/>
     </row>
-    <row r="32" ht="44.5" customHeight="1">
+    <row r="32" ht="31" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>AC19</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Each notification is delivered in the system as it is raised and appears in the recipient's notification list (see: View Notifications, SPM-71).</t>
+          <t>The Event Organiser who owns the event is notified when an Event Coordinator is assigned, with the Coordinator's name.</t>
         </is>
       </c>
       <c r="C32" s="8" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>SPM-53-TC01</t>
+          <t>SPM-53-TC02</t>
         </is>
       </c>
       <c r="F32" s="9" t="n"/>
@@ -1211,68 +1489,350 @@
     <row r="33" ht="17.5" customHeight="1">
       <c r="A33" s="11" t="inlineStr">
         <is>
-          <t>AC20</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Notifications are associated with the relevant event.</t>
+          <t>The newly assigned Coordinator is notified of the assignment.</t>
         </is>
       </c>
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>SPM-53-TC01</t>
+          <t>SPM-53-TC03</t>
         </is>
       </c>
       <c r="F33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="58" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>AC7</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Given an event is reassigned to a different Coordinator, when the reassignment is saved, then the newly assigned Coordinator and the Event Organiser are notified as for an assignment, and the previously assigned Coordinator is notified that the event is no longer theirs.</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC04</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="31" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>AC8</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Every active Venue Staff user is notified when a venue booking request is submitted for review.</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC08</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="44.5" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>AC9</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>The assigned Event Coordinator is notified when Venue Staff approve or reject a venue booking request for the event, with the venue, the requested times and, for a rejection, the reason.</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC09</t>
+        </is>
+      </c>
+      <c r="F36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="58" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>AC10</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Every active Technical Support Staff user is notified when the assigned Event Coordinator adds, removes or changes the quantity of an equipment requirement on an event in Planning or Confirmed (the events listed in the Equipment Requests queue, SPM-48).</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC10</t>
+        </is>
+      </c>
+      <c r="F37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="44.5" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>AC11</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>The assigned Event Coordinator is notified when Technical Support Staff mark an equipment requirement Reserved, Partially fulfilled or Cannot be provided.</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC11</t>
+        </is>
+      </c>
+      <c r="F38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="31" customHeight="1">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>AC12</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>The assigned Event Coordinator is notified when the Event Organiser submits a change request.</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC12</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n"/>
+    </row>
+    <row r="40" ht="31" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>AC13</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>The Event Organiser is notified of the outcome of a change request, including the outcome for each field where it is partially approved.</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC13</t>
+        </is>
+      </c>
+      <c r="F40" s="9" t="n"/>
+    </row>
+    <row r="41" ht="71.5" customHeight="1">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>AC14</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Given an important change (date and time, expected attendance, venue requirements or equipment) is saved by the assigned Coordinator or applied from an approved change request, when it is saved, then the Event Organiser who owns the event is notified, naming which of these changed. No other user is notified of the change by this criterion.</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC14</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n"/>
+    </row>
+    <row r="42" ht="44.5" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>AC15</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>The Event Organiser who owns the event is notified when the event moves from Confirmed back to Planning (an important change, SPM-62, or a safety check closed after a change, SPM-88).</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC15</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="n"/>
+    </row>
+    <row r="43" ht="58" customHeight="1">
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>AC16</t>
+        </is>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>An Attendee is notified when they are registered for an event, including when the Event Coordinator adds them (SPM-57), and when an event they are registered for is Postponed or Cancelled (see the confirmed, completed, postponed or cancelled criterion below).</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC17
+SPM-53-TC19</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n"/>
+    </row>
+    <row r="44" ht="31" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>AC17</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>Attendees whose registration is Registered are notified of the new date and time when an event is rescheduled.</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC16</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="n"/>
+    </row>
+    <row r="45" ht="58" customHeight="1">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>AC18</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>The Event Organiser who owns the event is notified when it is Confirmed, Completed, Postponed or Cancelled. Attendees whose registration is Registered are notified when it is Postponed or Cancelled. For Postponed and Cancelled, the notification includes the recorded reason.</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="n"/>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC18
+SPM-53-TC19</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n"/>
+    </row>
+    <row r="46" ht="44.5" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>AC19</t>
+        </is>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Each notification is delivered in the system as it is raised and appears in the recipient's notification list (see: View Notifications, SPM-71).</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC20</t>
+        </is>
+      </c>
+      <c r="F46" s="9" t="n"/>
+    </row>
+    <row r="47" ht="17.5" customHeight="1">
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>AC20</t>
+        </is>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>Notifications are associated with the relevant event.</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="n"/>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC21</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="B42:D42"/>
     <mergeCell ref="E33:F33"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="B44:D44"/>
     <mergeCell ref="B29:D29"/>
-    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="E44:F44"/>
     <mergeCell ref="B28:D28"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="E38:F38"/>
     <mergeCell ref="E29:F29"/>
-    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B40:D40"/>
     <mergeCell ref="E28:F28"/>
-    <mergeCell ref="E13:F13"/>
     <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="E40:F40"/>
     <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B24:D24"/>
     <mergeCell ref="E31:F31"/>
-    <mergeCell ref="B20:D20"/>
     <mergeCell ref="B33:D33"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="B36:D36"/>
     <mergeCell ref="E30:F30"/>
-    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="B41:D41"/>
     <mergeCell ref="B32:D32"/>
-    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B35:D35"/>
     <mergeCell ref="E27:F27"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="B47:D47"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="E32:F32"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="E41:F41"/>
     <mergeCell ref="B27:D27"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E37:F37"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="E47:F47"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1282,8 +1842,1902 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC09</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The assigned coordinator is notified of a booking approval and a rejection, with the venue, times and reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC08 has just been run. Run npm run fixtures:spm53 after this case.
+Logged in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="166" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Booking Requests' in the sidebar
+2. On the 'SPM53 Harbour Booking Review' card for SPM53 Hall, click 'Approve'
+3. In the dialog, click 'Approve'
+4. On the 'SPM53 Harbour Booking Review' card for SPM53 Studio, click 'Reject with a reason'
+5. In 'Reason for rejection', type the reason
+6. Leave 'Suggest another venue' on 'No venue suggested', then click 'Reject request'
+7. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+8. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Approve: SPM53 Hall (SPM53-HAL)
+Reject: SPM53 Studio (SPM53-STU), reason 'The studio is being repainted that week.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="125.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 3: A green 'Booking approved' message appears.
+Step 6: A green 'Booking request rejected' message appears.
+Step 8: Two unread notifications for 'SPM53 Harbour Booking Review' are listed, newest first: 'Venue booking rejected' ('SPM53 Studio (SPM53-STU) for "SPM53 Harbour Booking Review" on 23 Mar 2028, 09:00–12:00 was rejected. Reason: The studio is being repainted that week.') and 'Venue booking approved' ('SPM53 Hall (SPM53-HAL) for "SPM53 Harbour Booking Review" on 23 Mar 2028, 07:00–12:00 was approved.').</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC10</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Technical Support are notified when the coordinator adds, changes the quantity of and removes equipment</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 before this case. Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC11. 'SPM53 Harbour Equipment Fair' is in Planning, raised by Rachel Ng and assigned to Daniel Tan, with three Requested lines: SPM53 Projector × 2 (4 in stock), SPM53 Lectern Mic × 1 (2 in stock) and SPM53 Screen × 1. SPM53 Speaker has 2 in stock.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="206.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Equipment Fair'
+2. Click the 'Equipment' tab
+3. In 'Add equipment', choose 'SPM53 Speaker', set 'Quantity' to 1 and click 'Add'
+4. Change the 'Quantity' on the 'SPM53 Lectern Mic' row to 3 and click 'Save' on that row
+5. Click 'Remove' on the 'SPM53 Screen' row
+6. In the confirmation dialog, click 'Remove'
+7. Log out and log in as Technical Support Aisha Omar (aisha.omar@connectsphere.com / password123)
+8. Click 'Notifications' in the sidebar
+9. Log out and log in as Technical Support Vikram Nair (vikram.nair@connectsphere.com / password123)
+10. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Add: SPM53 Speaker × 1
+Change: SPM53 Lectern Mic 1 -&gt; 3
+Remove: SPM53 Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="179.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 3: A row for 'SPM53 Speaker' appears with Quantity 1 and status 'Requested'.
+Step 4: The 'Save' button disappears and the row shows Quantity 3.
+Step 6: The 'SPM53 Screen' row disappears.
+Step 8: Three unread notifications 'Equipment requirement changed' for 'SPM53 Harbour Equipment Fair' are listed, newest first: 'SPM53 Screen was removed from "SPM53 Harbour Equipment Fair".', 'SPM53 Lectern Mic on "SPM53 Harbour Equipment Fair" changed from 1 to 3.' and 'SPM53 Speaker × 1 was added to "SPM53 Harbour Equipment Fair".'
+Step 10: Vikram Nair's list has the same three notifications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The coordinator is notified when Technical Support mark lines Reserved, Partially fulfilled and Cannot be provided</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC10 has just been run. Run npm run fixtures:spm53 after this case.
+Logged in as Technical Support Vikram Nair (vikram.nair@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="166" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Equipment Requests' in the sidebar
+2. Open the equipment request for 'SPM53 Harbour Equipment Fair'
+3. Click 'Reserve' on the SPM53 Projector line
+4. Click 'Reserve' on the SPM53 Lectern Mic line
+5. On the SPM53 Speaker line, click 'Update'
+6. In 'Fulfilment status', choose 'Cannot be provided'
+7. In 'Technical notes', enter the notes
+8. Click 'Save'
+9. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+10. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Technical notes (SPM53 Speaker): Both speakers are booked for another event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="193" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 3: 'Reservation saved: 2 reserved.' appears and the line's status chip shows 'Reserved'.
+Step 4: 'Reservation saved: 2 reserved.' appears and the line's status chip shows 'Partially fulfilled'.
+Step 8: 'Update saved.' appears and the Status chip shows 'Cannot be provided'.
+Step 10: Three unread notifications for 'SPM53 Harbour Equipment Fair' are listed, newest first: 'Equipment cannot be provided' ('SPM53 Speaker for "SPM53 Harbour Equipment Fair" is now Cannot be provided.'), 'Equipment partially fulfilled' ('SPM53 Lectern Mic for "SPM53 Harbour Equipment Fair" is now Partially fulfilled.') and 'Equipment reserved' ('SPM53 Projector for "SPM53 Harbour Equipment Fair" is now Reserved.').</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The assigned coordinator is notified when the organiser sends a change request</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 before this case. Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC13. 'SPM53 Harbour Change Review' is in Planning, raised by Rachel Ng and assigned to Daniel Tan: Expected attendance 30, Description 'Quarterly briefing.', no change requests.
+Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="166" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'My Events' in the sidebar and open 'SPM53 Harbour Change Review'
+2. Click 'Request a change'
+3. Change 'Event name' to 'SPM53 Harbour Change Review and Lunch'
+4. Change 'Description' to 'Quarterly briefing with lunch.'
+5. Change 'Expected attendance' to 45
+6. Enter the reason in 'Reason for the change'
+7. Click 'Send change request'
+8. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+9. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Reason for the change: More clients have confirmed and we are adding lunch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 7: The change request is sent and listed on the event as Pending.
+Step 9: An unread notification 'Change request received' is listed with the message 'Rachel Ng has sent a change request for "SPM53 Harbour Change Review".' and the event 'SPM53 Harbour Change Review' with its reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A partly approved change request tells the organiser the outcome of each field</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC12 has just been run. Run npm run fixtures:spm53 after this case.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="139" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Change Requests' in the sidebar
+2. Click 'Review' on the request for 'SPM53 Harbour Change Review'
+3. For 'Event name', choose 'Reject' and enter the reason
+4. For 'Description' and 'Expected attendance', choose 'Approve'
+5. Click 'Save decision'
+6. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+7. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event name: reject, reason 'The invitations have already gone out.'
+Description and Expected attendance: approve</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="139" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 5: 'Change request processed.' is shown and the request is Partially approved.
+Step 7: An unread notification 'Change request partially approved' is listed with the message 'Your change request for "SPM53 Harbour Change Review" was partially approved. Event name: rejected – The invitations have already gone out. Description: approved. Expected attendance: approved.' Beside it, 'Event information changed' reads '"SPM53 Harbour Change Review" has changed: Expected attendance.' (the approved change applied, AC14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>An ordinary edit notifies nobody, and an important change tells the organiser which information changed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 before and after this case. 'SPM53 Harbour Edit Forum' is Approved, raised by Rachel Ng and assigned to Daniel Tan, Expected attendance 30, with no arrangements.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="247" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Edit Forum'
+2. Click 'Edit event information'
+3. Change 'Description' to the new description
+4. Click 'Save changes'
+5. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+6. Click 'Notifications' in the sidebar
+7. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+8. Click 'All Events' in the sidebar and open 'SPM53 Harbour Edit Forum'
+9. Click 'Edit event information'
+10. Change 'Expected attendance' to 50
+11. Click 'Save changes'
+12. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+13. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Description: Morning session with a networking break.
+Expected attendance: 30 -&gt; 50</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="139" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 4: The form is replaced by a green alert 'Event information updated.'
+Step 6: There is no notification about 'SPM53 Harbour Edit Forum'.
+Step 11: The form is replaced by a green alert 'Event information updated.'
+Step 13: An unread notification 'Event information changed' is listed with the message '"SPM53 Harbour Edit Forum" has changed: Expected attendance.' and the event 'SPM53 Harbour Edit Forum' with its reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC15</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Rescheduling a Confirmed event tells the organiser it changed and is no longer confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 before this case. Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC16. 'SPM53 Harbour Confirmed Gala' (18 Apr 2028, 09:00–12:00) is Confirmed, raised by Rachel Ng and assigned to Daniel Tan, with an Approved booking at SPM53 Hall and SPM53 Projector × 1 Reserved. Lee Wei Ming is Registered; Anita Devi has withdrawn.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="139" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Confirmed Gala'
+2. Click 'Edit event information'
+3. Change 'Starts at' to 25 Apr 2028, 09:00
+4. Change 'Ends at' to 25 Apr 2028, 12:00
+5. Click 'Save changes'
+6. Click 'Save and move to Planning'
+7. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+8. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Date: 18 Apr 2028, 09:00–12:00 -&gt; 25 Apr 2028, 09:00–12:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="152.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 5: The 'Move this event back to Planning?' dialog appears.
+Step 6: A green alert 'Event information updated. The event is back in Planning and needs to be confirmed again.' is shown.
+Step 8: Two unread notifications for 'SPM53 Harbour Confirmed Gala' are listed: 'Event information changed' ('"SPM53 Harbour Confirmed Gala" has changed: Date and time.') and 'Event no longer confirmed' ('"SPM53 Harbour Confirmed Gala" has moved back to Planning after a change and is no longer confirmed.').</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC16</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Only attendees whose registration is Registered are told the new date and time</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC15 has just been run. Run npm run fixtures:spm53 after this case.
+Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Log out and log in as Attendee Lee Wei Ming (lee.wei.ming@example.com / password123)
+2. Click 'Notifications' in the sidebar
+3. Log out and log in as Attendee Anita Devi (anita.devi@example.com / password123)
+4. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Registered: Lee Wei Ming
+Withdrawn: Anita Devi</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 2: An unread notification 'Event rescheduled' is listed with the message '"SPM53 Harbour Confirmed Gala" has a new date and time: 25 Apr 2028, 09:00–12:00.' and the event 'SPM53 Harbour Confirmed Gala' with its reference.
+Step 4: Anita Devi's list has no notification about 'SPM53 Harbour Confirmed Gala'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC17</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>An attendee who registers for an event is notified that they are registered</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 just before this case (it sets 'SPM53 Harbour Finished Dinner' to yesterday). Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC19. 'SPM53 Harbour Postponed Fair' is Confirmed with registration open; Lee Wei Ming is not registered.
+Logged in as Attendee Lee Wei Ming (lee.wei.ming@example.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Browse Events' in the sidebar
+2. Click 'SPM53 Harbour Postponed Fair'
+3. Click 'Register'
+4. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event: SPM53 Harbour Postponed Fair
+Attendee: Lee Wei Ming</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 3: A green alert 'You're registered for this event.' appears, with the status badge 'Registered'.
+Step 4: An unread notification 'Registration confirmed' is listed with the message 'You're registered for "SPM53 Harbour Postponed Fair".' and the event 'SPM53 Harbour Postponed Fair' with its reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC18</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>The organiser is notified when the coordinator confirms an event and marks one completed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC17 has just been run. 'SPM53 Harbour Ready Launch' is in Planning with an Approved booking and SPM53 Projector × 1 Reserved; 'SPM53 Harbour Finished Dinner' is Confirmed and ended yesterday evening (19:00–22:00). Both are Rachel Ng's, assigned to Daniel Tan.
+Logged in as Attendee Lee Wei Ming (lee.wei.ming@example.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="179.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+2. Click 'All Events' in the sidebar and open 'SPM53 Harbour Ready Launch'
+3. Click 'Confirm event'
+4. Click 'Confirm event' in the dialog
+5. Click 'All Events' in the sidebar and open 'SPM53 Harbour Finished Dinner'
+6. Click 'Mark as completed'
+7. Click 'Mark as completed' in the dialog
+8. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+9. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Confirm: SPM53 Harbour Ready Launch
+Complete: SPM53 Harbour Finished Dinner</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 4: The message 'The event is confirmed. The organiser can now see the arrangements.' is shown and the status badge changes to 'Confirmed'.
+Step 7: The status badge changes to 'Completed'.
+Step 9: Two new unread notifications are listed, newest first: 'Event completed' ('"SPM53 Harbour Finished Dinner" has been marked completed.') and 'Event confirmed' ('"SPM53 Harbour Ready Launch" is confirmed.').</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1320,7 +3774,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -1328,7 +3782,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Submitting a request notifies every Event Coordinator Lead, and assigning then reassigning it notifies each coordinator and the organiser</t>
+          <t>Submitting an event request notifies every active Event Coordinator Lead, naming the event</t>
         </is>
       </c>
     </row>
@@ -1340,12 +3794,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 before and after this case (it changes the SPM53 events and raises notifications). 'SPM53 Harbour Draft Summit' is a complete Draft of Rachel Ng's (Meridian Financial Group).
+          <t>Run npm run fixtures:spm53 before this case. Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC04. 'SPM53 Harbour Draft Summit' is a complete Draft of Rachel Ng's (Meridian Financial Group).
 Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="409" customHeight="1">
+    <row r="5" ht="139" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1359,25 +3813,11 @@
 4. Log out and log in as Event Coordinator Lead Nadia Rahman (nadia.rahman@connectsphere.com / password123)
 5. Click 'Notifications' in the sidebar
 6. Log out and log in as Event Coordinator Lead Grace Lim (grace.lim@connectsphere.com / password123)
-7. Click 'Notifications' in the sidebar
-8. Click the 'New event request submitted' notification for 'SPM53 Harbour Draft Summit'
-9. Click 'Assignments' in the sidebar
-10. On the 'SPM53 Harbour Draft Summit' row, choose 'Daniel Tan' in 'Assign to'
-11. Click 'Assign'
-12. Click the 'Active events' tab
-13. On the 'SPM53 Harbour Draft Summit' row, choose 'Priya Raj' in 'Reassign to'
-14. Click 'Reassign'
-15. Click 'Reassign' in the dialog
-16. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
-17. Click 'Notifications' in the sidebar
-18. Log out and log in as Event Coordinator Priya Raj (priya.raj@connectsphere.com / password123)
-19. Click 'Notifications' in the sidebar
-20. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-21. Click 'Notifications' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+7. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1386,12 +3826,11 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Event: SPM53 Harbour Draft Summit
-Event Coordinator Leads: Grace Lim, Nadia Rahman
-Assign to: Daniel Tan, then reassign to Priya Raj</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="382" customHeight="1">
+Event Coordinator Leads: Nadia Rahman, Grace Lim</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="98.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1400,14 +3839,572 @@
       <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Step 3: The event's page opens with the status badge 'Submitted'.
-Step 5: Nadia Rahman's list has an unread notification 'New event request submitted' with the message '"SPM53 Harbour Draft Summit" has been submitted and needs a coordinator assigned.' and the event 'SPM53 Harbour Draft Summit' with its reference.
-Step 7: Grace Lim's list has the same unread notification.
-Step 8: The event page for 'SPM53 Harbour Draft Summit' opens, with the status badge 'Submitted'.
-Step 11: 'SPM53 Harbour Draft Summit' leaves the 'Awaiting assignment' list.
-Step 15: The message '"SPM53 Harbour Draft Summit" has been reassigned from Daniel Tan to Priya Raj.' appears.
-Step 17: Daniel Tan's list has two unread notifications for 'SPM53 Harbour Draft Summit', newest first: 'An event has been reassigned' ('"SPM53 Harbour Draft Summit" has been reassigned to Priya Raj. You are no longer its coordinator.') and 'You have been assigned an event' ('You are now the coordinator for "SPM53 Harbour Draft Summit".').
-Step 19: Priya Raj's list has an unread 'You have been assigned an event' with the message 'You are now the coordinator for "SPM53 Harbour Draft Summit".'
-Step 21: Rachel Ng's list has two unread 'Coordinator assigned' notifications for 'SPM53 Harbour Draft Summit', newest first: 'Priya Raj is now the coordinator for "SPM53 Harbour Draft Summit".' and 'Daniel Tan is now the coordinator for "SPM53 Harbour Draft Summit".'</t>
+Step 5: An unread notification 'New event request submitted' is listed with the message '"SPM53 Harbour Draft Summit" has been submitted and needs a coordinator assigned.' and the event 'SPM53 Harbour Draft Summit' with its reference.
+Step 7: Grace Lim's list has the same unread notification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC19</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Postponing and cancelling notify the organiser and only the Registered attendees, with the reason when there is one</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC18 has just been run. Run npm run fixtures:spm53 after this case. 'SPM53 Harbour Postponed Fair': Lee Wei Ming Registered (SPM-53-TC17), Anita Devi withdrawn. 'SPM53 Harbour Cancelled Summit': Confirmed, Lee Wei Ming Registered, Anita Devi on the waiting list.
+Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="287.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+2. Click 'All Events' in the sidebar and open 'SPM53 Harbour Postponed Fair'
+3. Click 'Postpone event'
+4. Type the reason in 'Reason (optional)'
+5. Click 'Postpone event' in the dialog
+6. Click 'All Events' in the sidebar and open 'SPM53 Harbour Cancelled Summit'
+7. Click 'Cancel event'
+8. Leave 'Reason (optional)' empty
+9. Click 'Cancel event' in the dialog
+10. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+11. Click 'Notifications' in the sidebar
+12. Log out and log in as Attendee Lee Wei Ming (lee.wei.ming@example.com / password123)
+13. Click 'Notifications' in the sidebar
+14. Log out and log in as Attendee Anita Devi (anita.devi@example.com / password123)
+15. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Postponement reason: The keynote speaker is unwell.
+Cancellation reason: (empty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="152.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 5: The status badge changes to 'Postponed'.
+Step 9: The status badge changes to 'Cancelled'.
+Step 11: Two new unread notifications are listed, newest first: 'Event cancelled' ('"SPM53 Harbour Cancelled Summit" has been cancelled.', with no reason) and 'Event postponed' ('"SPM53 Harbour Postponed Fair" has been postponed. Reason: The keynote speaker is unwell.').
+Step 13: Lee Wei Ming's list has the same two unread notifications, above 'Registration confirmed'.
+Step 15: Anita Devi's list has no notification about 'SPM53 Harbour Postponed Fair' or 'SPM53 Harbour Cancelled Summit'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC20</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>A notification appears in the recipient's list, unread, as soon as it is raised</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 before this case. Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC21. 'SPM53 Harbour Live Update' is Under review, raised by Rachel Ng and assigned to Daniel Tan.
+Two browser windows: a normal one and a private one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="179.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. In the normal window, log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123) and click 'Notifications' in the sidebar
+2. In the private window, log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+3. In the private window, click 'Review Queue' in the sidebar and open 'SPM53 Harbour Live Update'
+4. Click 'Review request'
+5. Select 'Approve – planning can start'
+6. Click 'Approve request'
+7. Click 'Approve' in the dialog
+8. In the normal window, click 'Notifications' in the sidebar again</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event: SPM53 Harbour Live Update</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 1: Rachel Ng's Notifications page opens. Note the number on the bell at the top of the page (no number when nothing is unread).
+Step 7: A green 'Request approved' alert is shown.
+Step 8: 'Event request approved' ('"SPM53 Harbour Live Update" has been approved.') is at the top of the list, marked 'Unread', dated just now. The bell shows one more than in Step 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC21</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17.5" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Selecting a notification opens the event it is about</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC20 has just been run. Run npm run fixtures:spm53 after this case.
+Rachel Ng's Notifications page is open in the normal window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click the 'Event request approved' notification for 'SPM53 Harbour Live Update'
+2. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Event: SPM53 Harbour Live Update</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 1: The event page for 'SPM53 Harbour Live Update' opens on its Overview, with the status badge 'Approved'.
+Step 2: The 'Event request approved' notification is no longer marked 'Unread'.</t>
         </is>
       </c>
     </row>
@@ -1528,7 +4525,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -1536,11 +4533,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The organiser hears of a clarification request and of the approval or rejection, the coordinator hears it was answered, and nobody else is told the outcome</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="98.5" customHeight="1">
+          <t>Assigning a coordinator tells the organiser the coordinator's name</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1548,12 +4545,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 before and after this case (it changes the SPM53 events and raises notifications). 'SPM53 Harbour Clarity Forum' and 'SPM53 Harbour Rejected Brief' are Under review, raised by Rachel Ng and assigned to Daniel Tan, with no clarification open.
-Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="503.5" customHeight="1">
+          <t>SPM-53-TC01 has just been run.
+Logged in as Event Coordinator Lead Grace Lim (grace.lim@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="98.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1561,38 +4558,15 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Review Queue' in the sidebar and open 'SPM53 Harbour Clarity Forum'
-2. Click 'Review request'
-3. Choose 'Ask the organiser for clarification'
-4. Tick 'When' under 'What needs clarification'
-5. Type the message in 'Message to the organiser'
-6. Click 'Send request'
-7. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-8. Click 'Notifications' in the sidebar
-9. Click 'My Events' in the sidebar and open 'SPM53 Harbour Clarity Forum'
-10. Click 'Update request' in the 'Clarification requested' banner
-11. Replace 'Description' with the new description
-12. Click 'Resubmit request'
-13. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
-14. Click 'Notifications' in the sidebar
-15. Click 'Review Queue' in the sidebar and open 'SPM53 Harbour Clarity Forum'
-16. Click 'Review request'
-17. Select 'Approve – planning can start'
-18. Click 'Approve request'
-19. Click 'Approve' in the dialog
-20. Click 'Review Queue' in the sidebar and open 'SPM53 Harbour Rejected Brief'
-21. Click 'Review request'
-22. Select 'Reject this request'
-23. Type the reason into 'Reason for rejection'
-24. Click 'Reject request'
-25. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-26. Click 'Notifications' in the sidebar
-27. Log out and log in as Event Coordinator Lead Grace Lim (grace.lim@connectsphere.com / password123)
-28. Click 'Notifications' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+          <t>1. Click 'Assignments' in the sidebar
+2. On the 'SPM53 Harbour Draft Summit' row, choose 'Daniel Tan' in 'Assign to'
+3. Click 'Assign'
+4. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+5. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1600,13 +4574,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Message to the organiser: Can the forum start at 10:00 instead of 09:00?
-New description: The forum can start at 10:00; doors open at 09:30.
-Reason for rejection (SPM53 Harbour Rejected Brief): The brief duplicates the March town hall; please merge the two.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="328" customHeight="1">
+          <t>Event: SPM53 Harbour Draft Summit
+Assign to: Daniel Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1614,14 +4587,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 6: The clarification request is sent and the event stays Under review.
-Step 8: An unread notification 'Clarification requested' is listed with the message 'Your coordinator asked for clarification on "SPM53 Harbour Clarity Forum": Can the forum start at 10:00 instead of 09:00?' and the event 'SPM53 Harbour Clarity Forum' with its reference.
-Step 12: The event page opens with a green message 'Your updated request has been sent to Daniel Tan. It stays Under review.'
-Step 14: An unread notification 'Clarification answered' is listed with the message 'The organiser has responded to your clarification request on "SPM53 Harbour Clarity Forum".'
-Step 19: A green 'Request approved' alert is shown and the status badge changes to 'Approved'.
-Step 24: A green 'Request rejected' alert is shown and the status badge changes to 'Rejected'.
-Step 26: Two new unread notifications are listed, newest first: 'Event request rejected' ('"SPM53 Harbour Rejected Brief" has been rejected. Reason: The brief duplicates the March town hall; please merge the two.') and 'Event request approved' ('"SPM53 Harbour Clarity Forum" has been approved.').
-Step 28: Grace Lim's list has no 'Event request approved' or 'Event request rejected' notification for either event.</t>
+          <t>Step 3: 'SPM53 Harbour Draft Summit' leaves the 'Awaiting assignment' list.
+Step 5: An unread notification 'Coordinator assigned' is listed with the message 'Daniel Tan is now the coordinator for "SPM53 Harbour Draft Summit".' and the event 'SPM53 Harbour Draft Summit' with its reference.</t>
         </is>
       </c>
     </row>
@@ -1742,7 +4709,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="17.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -1750,11 +4717,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A venue booking request notifies every Venue Staff user, and the coordinator hears each approval and rejection with the venue, times and reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="112" customHeight="1">
+          <t>The newly assigned coordinator is notified of the assignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1762,12 +4729,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 before and after this case (it changes the SPM53 events and raises notifications). 'SPM53 Harbour Booking Review' (23 Mar 2028, 09:00–12:00) is in Planning, assigned to Daniel Tan, with one Pending request for SPM53 Studio (SPM53-STU). SPM53 Hall (SPM53-HAL) is free that day.
-Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="328" customHeight="1">
+          <t>SPM-53-TC02 has just been run.
+Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1775,27 +4742,12 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Booking Review'
-2. Click the 'Venue' tab
-3. Click 'Request booking' on SPM53 Hall
-4. Leave only 'AM (07:00–12:00)' ticked
-5. Click 'Submit request'
-6. Log out and log in as Venue Staff Siti Hassan (siti.hassan@connectsphere.com / password123)
-7. Click 'Notifications' in the sidebar
-8. Log out and log in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123)
-9. Click 'Notifications' in the sidebar
-10. Click 'Booking Requests' in the sidebar
-11. On the 'SPM53 Harbour Booking Review' card for SPM53 Hall, click 'Approve'
-12. In the dialog, click 'Approve'
-13. On the 'SPM53 Harbour Booking Review' card for SPM53 Studio, click 'Reject with a reason'
-14. In 'Reason for rejection', type the reason
-15. Leave 'Suggest another venue' on 'No venue suggested', then click 'Reject request'
-16. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
-17. Click 'Notifications' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>1. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+2. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1803,13 +4755,11 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM53 Harbour Booking Review
-New request: SPM53 Hall (SPM53-HAL), 23 Mar 2028, AM
-Reject: SPM53 Studio (SPM53-STU), reason 'The studio is being repainted that week.'</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="220" customHeight="1">
+          <t>Coordinator: Daniel Tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="44.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1817,12 +4767,7 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 5: 'Booking request sent to Venue Staff.' is shown.
-Step 7: Siti Hassan's list has an unread notification 'Venue booking request to review' with the message '"SPM53 Harbour Booking Review" requests SPM53 Hall (SPM53-HAL) on 23 Mar 2028, 07:00–12:00.' and the event 'SPM53 Harbour Booking Review' with its reference.
-Step 9: Marcus Wong's list has the same unread notification.
-Step 12: A green 'Booking approved' message appears.
-Step 15: A green 'Booking request rejected' message appears.
-Step 17: Two unread notifications for 'SPM53 Harbour Booking Review' are listed, newest first: 'Venue booking rejected' ('SPM53 Studio (SPM53-STU) for "SPM53 Harbour Booking Review" on 23 Mar 2028, 09:00–12:00 was rejected. Reason: The studio is being repainted that week.') and 'Venue booking approved' ('SPM53 Hall (SPM53-HAL) for "SPM53 Harbour Booking Review" on 23 Mar 2028, 07:00–12:00 was approved.').</t>
+          <t>Step 2: An unread notification 'You have been assigned an event' is listed with the message 'You are now the coordinator for "SPM53 Harbour Draft Summit".'</t>
         </is>
       </c>
     </row>
@@ -1951,11 +4896,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Equipment added, changed and removed notifies Technical Support and the organiser, and each fulfilment outcome notifies the coordinator</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="112" customHeight="1">
+          <t>Reassigning notifies the new coordinator and the organiser, and tells the previous coordinator the event is no longer theirs</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1963,12 +4908,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 before and after this case (it changes the SPM53 events and raises notifications). 'SPM53 Harbour Equipment Fair' is in Planning, raised by Rachel Ng and assigned to Daniel Tan, with three Requested lines: SPM53 Projector × 2 (4 in stock), SPM53 Lectern Mic × 1 (2 in stock) and SPM53 Screen × 1. SPM53 Speaker has 2 in stock.
+          <t>SPM-53-TC03 has just been run. Run npm run fixtures:spm53 after this case.
 Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="409" customHeight="1">
+    <row r="5" ht="233.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1976,32 +4921,22 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Equipment Fair'
-2. Click the 'Equipment' tab
-3. In 'Add equipment', choose 'SPM53 Speaker', set 'Quantity' to 1 and click 'Add'
-4. Change the 'Quantity' on the 'SPM53 Lectern Mic' row to 3 and click 'Save' on that row
-5. Click 'Remove' on the 'SPM53 Screen' row
-6. In the confirmation dialog, click 'Remove'
-7. Log out and log in as Technical Support Aisha Omar (aisha.omar@connectsphere.com / password123)
+          <t>1. Log out and log in as Event Coordinator Lead Grace Lim (grace.lim@connectsphere.com / password123)
+2. Click 'Assignments' in the sidebar
+3. Click the 'Active events' tab
+4. On the 'SPM53 Harbour Draft Summit' row, choose 'Priya Raj' in 'Reassign to'
+5. Click 'Reassign'
+6. Click 'Reassign' in the dialog
+7. Log out and log in as Event Coordinator Priya Raj (priya.raj@connectsphere.com / password123)
 8. Click 'Notifications' in the sidebar
-9. Log out and log in as Technical Support Vikram Nair (vikram.nair@connectsphere.com / password123)
+9. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
 10. Click 'Notifications' in the sidebar
-11. Click 'Equipment Requests' in the sidebar
-12. Open the equipment request for 'SPM53 Harbour Equipment Fair'
-13. Click 'Reserve' on the SPM53 Projector line
-14. Click 'Reserve' on the SPM53 Lectern Mic line
-15. On the SPM53 Speaker line, click 'Update'
-16. In 'Fulfilment status', choose 'Cannot be provided'
-17. In 'Technical notes', enter the notes
-18. Click 'Save'
-19. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
-20. Click 'Notifications' in the sidebar
-21. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-22. Click 'Notifications' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="85" customHeight="1">
+11. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+12. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2009,15 +4944,13 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM53 Harbour Equipment Fair
-Add: SPM53 Speaker × 1
-Change: SPM53 Lectern Mic 1 -&gt; 3
-Remove: SPM53 Screen
-Technical notes (SPM53 Speaker): Both speakers are booked for another event.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="422.5" customHeight="1">
+          <t>Event: SPM53 Harbour Draft Summit
+From: Daniel Tan
+To: Priya Raj</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="179.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2025,16 +4958,10 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 3: A row for 'SPM53 Speaker' appears with Quantity 1 and status 'Requested'.
-Step 4: The 'Save' button disappears and the row shows Quantity 3.
-Step 6: The 'SPM53 Screen' row disappears.
-Step 8: Aisha Omar's list has three unread notifications 'Equipment requirement changed' for 'SPM53 Harbour Equipment Fair', newest first: 'SPM53 Screen was removed from "SPM53 Harbour Equipment Fair".', 'SPM53 Lectern Mic on "SPM53 Harbour Equipment Fair" changed from 1 to 3.' and 'SPM53 Speaker × 1 was added to "SPM53 Harbour Equipment Fair".'
-Step 10: Vikram Nair's list has the same three notifications.
-Step 13: 'Reservation saved: 2 reserved.' appears and the line's status chip shows 'Reserved'.
-Step 14: 'Reservation saved: 2 reserved.' appears and the line's status chip shows 'Partially fulfilled'.
-Step 18: 'Update saved.' appears and the Status chip shows 'Cannot be provided'.
-Step 20: Three unread notifications for 'SPM53 Harbour Equipment Fair' are listed, newest first: 'Equipment cannot be provided' ('SPM53 Speaker for "SPM53 Harbour Equipment Fair" is now Cannot be provided.'), 'Equipment partially fulfilled' ('SPM53 Lectern Mic for "SPM53 Harbour Equipment Fair" is now Partially fulfilled.') and 'Equipment reserved' ('SPM53 Projector for "SPM53 Harbour Equipment Fair" is now Reserved.').
-Step 22: Three unread notifications 'Event information changed' for 'SPM53 Harbour Equipment Fair' are listed, each with the message '"SPM53 Harbour Equipment Fair" has changed: Equipment requirements.'</t>
+          <t>Step 6: The message '"SPM53 Harbour Draft Summit" has been reassigned from Daniel Tan to Priya Raj.' appears.
+Step 8: An unread notification 'You have been assigned an event' is listed with the message 'You are now the coordinator for "SPM53 Harbour Draft Summit".'
+Step 10: An unread notification 'An event has been reassigned' is listed with the message '"SPM53 Harbour Draft Summit" has been reassigned to Priya Raj. You are no longer its coordinator.'
+Step 12: A new unread 'Coordinator assigned' notification reads 'Priya Raj is now the coordinator for "SPM53 Harbour Draft Summit".', above the one naming Daniel Tan from SPM-53-TC02.</t>
         </is>
       </c>
     </row>
@@ -2155,7 +5082,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -2163,7 +5090,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A change request notifies the coordinator, and a partly approved decision tells the organiser each field's outcome and that the expected attendance changed</t>
+          <t>The organiser is notified when the assigned coordinator asks for clarification, with the message</t>
         </is>
       </c>
     </row>
@@ -2175,12 +5102,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 before and after this case (it changes the SPM53 events and raises notifications). 'SPM53 Harbour Change Review' is in Planning, raised by Rachel Ng and assigned to Daniel Tan: Expected attendance 30, Description 'Quarterly briefing.', no change requests.
-Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="301" customHeight="1">
+          <t>Run npm run fixtures:spm53 before this case. Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC07. 'SPM53 Harbour Clarity Forum' and 'SPM53 Harbour Rejected Brief' are Under review, raised by Rachel Ng and assigned to Daniel Tan.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="139" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2188,26 +5115,18 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'My Events' in the sidebar and open 'SPM53 Harbour Change Review'
-2. Click 'Request a change'
-3. Change 'Event name' to 'SPM53 Harbour Change Review and Lunch'
-4. Change 'Description' to 'Quarterly briefing with lunch.'
-5. Change 'Expected attendance' to 45
-6. Enter the reason in 'Reason for the change'
-7. Click 'Send change request'
-8. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
-9. Click 'Notifications' in the sidebar
-10. Click 'Change Requests' in the sidebar
-11. Click 'Review' on the request for 'SPM53 Harbour Change Review'
-12. For 'Event name', choose 'Reject' and enter the reason
-13. For 'Description' and 'Expected attendance', choose 'Approve'
-14. Click 'Save decision'
-15. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-16. Click 'Notifications' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="71.5" customHeight="1">
+          <t>1. Click 'Review Queue' in the sidebar and open 'SPM53 Harbour Clarity Forum'
+2. Click 'Review request'
+3. Choose 'Ask the organiser for clarification'
+4. Tick 'When' under 'What needs clarification'
+5. Type the message in 'Message to the organiser'
+6. Click 'Send request'
+7. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+8. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2215,13 +5134,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Reason for the change: More clients have confirmed and we are adding lunch.
-Event name: reject, reason 'The invitations have already gone out.'
-Description and Expected attendance: approve</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="220" customHeight="1">
+          <t>Event: SPM53 Harbour Clarity Forum
+Message to the organiser: Can the forum start at 10:00 instead of 09:00?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="98.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2229,10 +5147,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 7: The change request is sent and listed on the event as Pending.
-Step 9: An unread notification 'Change request received' is listed with the message 'Rachel Ng has sent a change request for "SPM53 Harbour Change Review".' and the event 'SPM53 Harbour Change Review' with its reference.
-Step 14: 'Change request processed.' is shown and the request is Partially approved.
-Step 16: Two new unread notifications for 'SPM53 Harbour Change Review' are listed: 'Change request partially approved' with the message 'Your change request for "SPM53 Harbour Change Review" was partially approved. Event name: rejected – The invitations have already gone out. Description: approved. Expected attendance: approved.', and 'Event information changed' with the message '"SPM53 Harbour Change Review" has changed: Expected attendance.'</t>
+          <t>Step 6: The clarification request is sent and the event stays Under review.
+Step 8: An unread notification 'Clarification requested' is listed with the message 'Your coordinator asked for clarification on "SPM53 Harbour Clarity Forum": Can the forum start at 10:00 instead of 09:00?' and the event 'SPM53 Harbour Clarity Forum' with its reference.</t>
         </is>
       </c>
     </row>
@@ -2353,7 +5269,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -2361,11 +5277,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>An ordinary edit notifies nobody; rescheduling a Confirmed event tells the organiser it changed and is no longer confirmed, and tells only Registered attendees the new date</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="112" customHeight="1">
+          <t>The assigned coordinator is notified when the organiser answers the clarification by resubmitting</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2373,12 +5289,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 before and after this case (it changes the SPM53 events and raises notifications). 'SPM53 Harbour Confirmed Gala' (18 Apr 2028, 09:00–12:00) is Confirmed, raised by Rachel Ng and assigned to Daniel Tan, with an Approved booking at SPM53 Hall and SPM53 Projector × 1 Reserved. Lee Wei Ming is Registered; Anita Devi has withdrawn.
-Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="355" customHeight="1">
+          <t>SPM-53-TC05 has just been run.
+Logged in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="125.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2386,29 +5302,16 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Confirmed Gala'
-2. Click 'Edit event information'
-3. Change 'Description' to the new description
-4. Click 'Save changes'
-5. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-6. Click 'Notifications' in the sidebar
-7. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
-8. Click 'All Events' in the sidebar and open 'SPM53 Harbour Confirmed Gala'
-9. Click 'Edit event information'
-10. Change 'Starts at' to 25 Apr 2028, 09:00
-11. Change 'Ends at' to 25 Apr 2028, 12:00
-12. Click 'Save changes'
-13. Click 'Save and move to Planning'
-14. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-15. Click 'Notifications' in the sidebar
-16. Log out and log in as Attendee Lee Wei Ming (lee.wei.ming@example.com / password123)
-17. Click 'Notifications' in the sidebar
-18. Log out and log in as Attendee Anita Devi (anita.devi@example.com / password123)
-19. Click 'Notifications' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+          <t>1. Click 'My Events' in the sidebar and open 'SPM53 Harbour Clarity Forum'
+2. Click 'Update request' in the 'Clarification requested' banner
+3. Replace 'Description' with the new description
+4. Click 'Resubmit request'
+5. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
+6. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2416,14 +5319,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Description: Gala dinner with an awards segment.
-Date: 18 Apr 2028, 09:00–12:00 -&gt; 25 Apr 2028, 09:00–12:00
-Registered: Lee Wei Ming
-Withdrawn: Anita Devi</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="287.5" customHeight="1">
+          <t>Event: SPM53 Harbour Clarity Forum
+Description: The forum can start at 10:00; doors open at 09:30.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2431,13 +5332,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 4: The form is replaced by a green alert 'Event information updated.' The event stays Confirmed.
-Step 6: There is no notification about 'SPM53 Harbour Confirmed Gala'.
-Step 12: The 'Move this event back to Planning?' dialog appears.
-Step 13: A green alert 'Event information updated. The event is back in Planning and needs to be confirmed again.' is shown.
-Step 15: Two unread notifications for 'SPM53 Harbour Confirmed Gala' are listed: 'Event information changed' ('"SPM53 Harbour Confirmed Gala" has changed: Date and time.') and 'Event no longer confirmed' ('"SPM53 Harbour Confirmed Gala" has moved back to Planning after a change and is no longer confirmed.').
-Step 17: An unread notification 'Event rescheduled' is listed with the message '"SPM53 Harbour Confirmed Gala" has a new date and time: 25 Apr 2028, 09:00–12:00.' and the event 'SPM53 Harbour Confirmed Gala' with its reference.
-Step 19: Anita Devi's list has no notification about 'SPM53 Harbour Confirmed Gala'.</t>
+          <t>Step 4: The event page opens with a green message 'Your updated request has been sent to Daniel Tan. It stays Under review.'
+Step 6: An unread notification 'Clarification answered' is listed with the message 'The organiser has responded to your clarification request on "SPM53 Harbour Clarity Forum".'</t>
         </is>
       </c>
     </row>
@@ -2558,7 +5454,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="58" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -2566,11 +5462,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Registering notifies the attendee; confirming, completing, postponing and cancelling notify the organiser, and postponing and cancelling notify only Registered attendees, with any reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="206.5" customHeight="1">
+          <t>An approval and a rejection notify only the organiser, the rejection with its reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2578,16 +5474,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Run npm run fixtures:spm53 just before this case, and again after it (it changes the SPM53 events, and sets 'SPM53 Harbour Finished Dinner' to yesterday on every run). All four events are raised by Rachel Ng and assigned to Daniel Tan:
-- 'SPM53 Harbour Ready Launch': Planning, with an Approved booking at SPM53 Studio and SPM53 Projector × 1 Reserved.
-- 'SPM53 Harbour Finished Dinner': Confirmed, ended yesterday evening (19:00–22:00).
-- 'SPM53 Harbour Postponed Fair': Confirmed, registration open; Anita Devi has withdrawn, Lee Wei Ming is not registered.
-- 'SPM53 Harbour Cancelled Summit': Confirmed; Lee Wei Ming is Registered, Anita Devi is on the waiting list.
-Logged in as Attendee Lee Wei Ming (lee.wei.ming@example.com / password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="449.5" customHeight="1">
+          <t>SPM-53-TC06 has just been run. Run npm run fixtures:spm53 after this case.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="247" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2595,31 +5487,210 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Browse Events' in the sidebar
-2. Click 'SPM53 Harbour Postponed Fair'
-3. Click 'Register'
-4. Click 'Notifications' in the sidebar
-5. Log out and log in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123)
-6. Click 'All Events' in the sidebar and open 'SPM53 Harbour Ready Launch'
-7. Click 'Confirm event'
-8. Click 'Confirm event' in the dialog
-9. Click 'All Events' in the sidebar and open 'SPM53 Harbour Finished Dinner'
-10. Click 'Mark as completed'
-11. Click 'Mark as completed' in the dialog
-12. Click 'All Events' in the sidebar and open 'SPM53 Harbour Postponed Fair'
-13. Click 'Postpone event'
-14. Type the reason in 'Reason (optional)'
-15. Click 'Postpone event' in the dialog
-16. Click 'All Events' in the sidebar and open 'SPM53 Harbour Cancelled Summit'
-17. Click 'Cancel event'
-18. Leave 'Reason (optional)' empty
-19. Click 'Cancel event' in the dialog
-20. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
-21. Click 'Notifications' in the sidebar
-22. Log out and log in as Attendee Lee Wei Ming (lee.wei.ming@example.com / password123)
-23. Click 'Notifications' in the sidebar
-24. Log out and log in as Attendee Anita Devi (anita.devi@example.com / password123)
-25. Click 'Notifications' in the sidebar</t>
+          <t>1. Click 'Review Queue' in the sidebar and open 'SPM53 Harbour Clarity Forum'
+2. Click 'Review request'
+3. Select 'Approve – planning can start'
+4. Click 'Approve request'
+5. Click 'Approve' in the dialog
+6. Click 'Review Queue' in the sidebar and open 'SPM53 Harbour Rejected Brief'
+7. Click 'Review request'
+8. Select 'Reject this request'
+9. Type the reason into 'Reason for rejection'
+10. Click 'Reject request'
+11. Log out and log in as Event Organiser Rachel Ng (rachel.ng@meridianfina.com / password123)
+12. Click 'Notifications' in the sidebar
+13. Log out and log in as Event Coordinator Lead Grace Lim (grace.lim@connectsphere.com / password123)
+14. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Approve: SPM53 Harbour Clarity Forum
+Reject: SPM53 Harbour Rejected Brief, reason 'The brief duplicates the March town hall; please merge the two.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="152.5" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 5: A green 'Request approved' alert is shown and the status badge changes to 'Approved'.
+Step 10: A green 'Request rejected' alert is shown and the status badge changes to 'Rejected'.
+Step 12: Two new unread notifications are listed, newest first: 'Event request rejected' ('"SPM53 Harbour Rejected Brief" has been rejected. Reason: The brief duplicates the March town hall; please merge the two.') and 'Event request approved' ('"SPM53 Harbour Clarity Forum" has been approved.').
+Step 14: Grace Lim's list has no 'Event request approved' or 'Event request rejected' notification for either event.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46324</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC08</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Sending a venue booking request notifies every active Venue Staff user</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="112" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 before this case. Do not run it again afterwards: go straight on to the next case(s), and reset after SPM-53-TC09. 'SPM53 Harbour Booking Review' (23 Mar 2028, 09:00–12:00) is in Planning, assigned to Daniel Tan, with one Pending request for SPM53 Studio (SPM53-STU). SPM53 Hall (SPM53-HAL) is free that day.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="166" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Booking Review'
+2. Click the 'Venue' tab
+3. Click 'Request booking' on SPM53 Hall
+4. Leave only 'AM (07:00–12:00)' ticked
+5. Click 'Submit request'
+6. Log out and log in as Venue Staff Siti Hassan (siti.hassan@connectsphere.com / password123)
+7. Click 'Notifications' in the sidebar
+8. Log out and log in as Venue Staff Marcus Wong (marcus.wong@connectsphere.com / password123)
+9. Click 'Notifications' in the sidebar</t>
         </is>
       </c>
     </row>
@@ -2631,12 +5702,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Postponement reason: The keynote speaker is unwell.
-Cancellation reason: (empty)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="328" customHeight="1">
+          <t>Event: SPM53 Harbour Booking Review
+Venue: SPM53 Hall (SPM53-HAL), 23 Mar 2028, AM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="98.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2644,15 +5715,9 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 3: A green alert 'You're registered for this event.' appears, with the status badge 'Registered'.
-Step 4: An unread notification 'Registration confirmed' is listed with the message 'You're registered for "SPM53 Harbour Postponed Fair".' and the event 'SPM53 Harbour Postponed Fair' with its reference.
-Step 8: The message 'The event is confirmed. The organiser can now see the arrangements.' is shown and the status badge changes to 'Confirmed'.
-Step 11: The status badge changes to 'Completed'.
-Step 15: The status badge changes to 'Postponed'.
-Step 19: The status badge changes to 'Cancelled'.
-Step 21: Four new unread notifications are listed, newest first: 'Event cancelled' ('"SPM53 Harbour Cancelled Summit" has been cancelled.', with no reason), 'Event postponed' ('"SPM53 Harbour Postponed Fair" has been postponed. Reason: The keynote speaker is unwell.'), 'Event completed' ('"SPM53 Harbour Finished Dinner" has been marked completed.') and 'Event confirmed' ('"SPM53 Harbour Ready Launch" is confirmed.').
-Step 23: Lee Wei Ming's list has the same unread 'Event cancelled' and 'Event postponed' notifications, above 'Registration confirmed'.
-Step 25: Anita Devi's list has no notification about 'SPM53 Harbour Postponed Fair' or 'SPM53 Harbour Cancelled Summit'.</t>
+          <t>Step 5: 'Booking request sent to Venue Staff.' is shown.
+Step 7: An unread notification 'Venue booking request to review' is listed with the message '"SPM53 Harbour Booking Review" requests SPM53 Hall (SPM53-HAL) on 23 Mar 2028, 07:00–12:00.' and the event 'SPM53 Harbour Booking Review' with its reference.
+Step 9: Marcus Wong's list has the same unread notification.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SPM-53: Notify the attendee the coordinator adds (AC16)
With SPM-57 merged, POST /api/events/[id]/registrations sends the same
"Registration confirmed" notification as self-registration to the attendee
it adds or re-adds, in the same transaction. New manual case SPM-53-TC22
on SPM53 Harbour Confirmed Gala; no new fixtures.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-53_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-53_Test_Cases.xlsx
@@ -28,6 +28,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC19" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC20" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC21" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC22" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -536,6 +537,7 @@
       <c r="H1" s="15" t="n"/>
       <c r="I1" s="14" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -1402,6 +1404,46 @@
       <c r="H24" s="13" t="n"/>
       <c r="I24" s="13" t="n"/>
     </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>TC22</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>SPM-53-TC22</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>An attendee the coordinator adds is notified that they are registered</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>AC16</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G25" s="13" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+    </row>
+    <row r="26"/>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
@@ -1738,7 +1780,8 @@
       <c r="E43" s="13" t="inlineStr">
         <is>
           <t>SPM-53-TC17
-SPM-53-TC19</t>
+SPM-53-TC19
+SPM-53-TC22</t>
         </is>
       </c>
       <c r="F43" s="14" t="n"/>
@@ -2225,6 +2268,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2423,6 +2467,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3016,6 +3061,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3403,6 +3449,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3594,6 +3641,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3791,6 +3839,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4183,6 +4232,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4558,6 +4608,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4622,6 +4673,193 @@
           <t>240f4cb</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="13" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>SPM-53-TC22</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17.5" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>An attendee the coordinator adds is notified that they are registered</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44.5" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Run npm run fixtures:spm53 before and after this case. 'SPM53 Harbour Confirmed Gala' is Confirmed with registration on and an Approved booking at SPM53 Hall (theatre, 60 seats), assigned to Daniel Tan. Anita Devi has withdrawn from it.
+Logged in as Event Coordinator Daniel Tan (daniel.tan@connectsphere.com / password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>1. Click 'All Events' in the sidebar and open 'SPM53 Harbour Confirmed Gala'
+2. Click the 'Attendees' tab
+3. Click 'Add attendee'
+4. Type the email in 'Attendee email'
+5. Click 'Add attendee' in the 'Add an attendee' form
+6. Log out and log in as Attendee Anita Devi (anita.devi@example.com / password123)
+7. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.5" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Event: SPM53 Harbour Confirmed Gala
+Attendee email: anita.devi@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Step 5: A green alert 'Anita Devi has been added to the registration list.' is shown, and Anita Devi is listed as Registered with 'Added by Daniel Tan'.
+Step 7: An unread notification 'Registration confirmed' is listed with the message 'You're registered for "SPM53 Harbour Confirmed Gala".' and the event 'SPM53 Harbour Confirmed Gala' with its reference.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>46325</v>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="12.5" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13" ht="12.5" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14" ht="12.5" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15" ht="12.5" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16" ht="12.5" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17" ht="12.5" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4750,6 +4988,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4929,6 +5168,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5123,6 +5363,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5511,6 +5752,7 @@
         <v>46324</v>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
SPM-53: Record the test case run (22 pass) and refresh the matrix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-53_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-53_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="11370" tabRatio="904" firstSheet="10" activeTab="15" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="904" firstSheet="6" activeTab="22" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -37,8 +37,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -192,7 +193,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,6 +227,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,7 +539,6 @@
       <c r="H1" s="15" t="n"/>
       <c r="I1" s="14" t="n"/>
     </row>
-    <row r="2"/>
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -1404,7 +1405,7 @@
       <c r="H24" s="13" t="n"/>
       <c r="I24" s="13" t="n"/>
     </row>
-    <row r="25">
+    <row r="25" ht="25" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>TC22</t>
@@ -1443,7 +1444,6 @@
       <c r="H25" s="13" t="n"/>
       <c r="I25" s="13" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27" ht="13" customHeight="1">
       <c r="A27" s="16" t="inlineStr">
         <is>
@@ -1877,8 +1877,8 @@
     <mergeCell ref="B29:D29"/>
     <mergeCell ref="E39:F39"/>
     <mergeCell ref="B38:D38"/>
+    <mergeCell ref="B34:D34"/>
     <mergeCell ref="E44:F44"/>
-    <mergeCell ref="B34:D34"/>
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="E35:F35"/>
     <mergeCell ref="B37:D37"/>
@@ -2066,7 +2066,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2082,7 +2082,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 3: A green 'Booking approved' message appears.
+Step 6: A green 'Booking request rejected' message appears.
+Step 8: Two unread notifications for 'SPM53 Harbour Booking Review' are listed, newest first: 'Venue booking rejected' ('SPM53 Studio (SPM53-STU) for "SPM53 Harbour Booking Review" on 23 Mar 2028, 09:00–12:00 was rejected. Reason: The studio is being repainted that week.') and 'Venue booking approved' ('SPM53 Hall (SPM53-HAL) for "SPM53 Harbour Booking Review" on 23 Mar 2028, 09:00–12:00 was approved.').</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2102,7 +2108,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -2110,7 +2120,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2118,7 +2132,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -2268,7 +2284,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2284,7 +2300,15 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 3: A row for 'SPM53 Speaker' appears with Quantity 1 and status 'Requested'.
+Step 4: The 'Save' button disappears and the row shows Quantity 3.
+Step 6: The 'SPM53 Screen' row disappears.
+Step 8: Three unread notifications 'Equipment requirement changed' for 'SPM53 Harbour Equipment Fair' are listed, newest first: 'SPM53 Screen was removed from "SPM53 Harbour Equipment Fair".', 'SPM53 Lectern Mic on "SPM53 Harbour Equipment Fair" changed from 1 to 3.' and 'SPM53 Speaker × 1 was added to "SPM53 Harbour Equipment Fair".'
+Step 10: Vikram Nair's list has the same three notifications.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2294,7 +2318,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2328,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -2312,7 +2340,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2320,7 +2352,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -2467,7 +2501,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2483,7 +2517,14 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 3: 'Reservation saved: 2 reserved.' appears and the line's status chip shows 'Reserved'.
+Step 4: 'Reservation saved: 2 reserved.' appears and the line's status chip shows 'Partially fulfilled'.
+Step 8: 'Update saved.' appears and the Status chip shows 'Cannot be provided'.
+Step 10: Three unread notifications for 'SPM53 Harbour Equipment Fair' are listed, newest first: 'Equipment cannot be provided' ('SPM53 Speaker for "SPM53 Harbour Equipment Fair" is now Cannot be provided.'), 'Equipment partially fulfilled' ('SPM53 Lectern Mic for "SPM53 Harbour Equipment Fair" is now Partially fulfilled.') and 'Equipment reserved' ('SPM53 Projector for "SPM53 Harbour Equipment Fair" is now Reserved.').</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2493,7 +2534,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2544,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -2511,7 +2556,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2519,7 +2568,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -2663,7 +2714,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2679,7 +2730,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 7: A green alert 'Change request sent to your coordinator.' is shown.
+Step 9: An unread notification 'Change request received' is listed with the message 'Rachel Ng has sent a change request for "SPM53 Harbour Change Review".' and the event 'SPM53 Harbour Change Review' with its reference.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2689,7 +2745,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -2699,7 +2755,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -2707,7 +2767,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2715,7 +2779,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -2858,7 +2924,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -2874,7 +2940,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 5: A green alert 'Change request processed.' is shown.
+Step 7: An unread notification 'Change request partially approved' is listed with the message 'Your change request for "SPM53 Harbour Change Review" was partially approved. Event name: rejected – The invitations have already gone out. Description: approved. Expected attendance: approved.' Beside it, 'Event information changed' reads '"SPM53 Harbour Change Review" has changed: Expected attendance.' (the approved change applied, AC14).</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -2884,7 +2955,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2965,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -2902,7 +2977,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -2910,7 +2989,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3061,7 +3142,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3077,7 +3158,14 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 4: The form is replaced by a green alert 'Event information updated.'
+Step 6: There is no notification about 'SPM53 Harbour Edit Forum'.
+Step 11: The form is replaced by a green alert 'Event information updated.'
+Step 13: An unread notification 'Event information changed' is listed with the message '"SPM53 Harbour Edit Forum" has changed: Expected attendance.' and the event 'SPM53 Harbour Edit Forum' with its reference.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -3087,7 +3175,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -3097,7 +3185,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -3105,7 +3197,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -3113,7 +3209,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3257,7 +3355,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3273,7 +3371,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 5: The 'Move this event back to Planning?' dialog appears.
+Step 6: A green alert 'Event information updated. The event is back in Planning and needs to be submitted for a safety check again.' is shown.
+Step 8: Two unread notifications for 'SPM53 Harbour Confirmed Gala' are listed: 'Event information changed' ('"SPM53 Harbour Confirmed Gala" has changed: Date and time.') and 'Event no longer confirmed' ('"SPM53 Harbour Confirmed Gala" has moved back to Planning after a change and is no longer confirmed.').</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -3283,7 +3387,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3397,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -3301,7 +3409,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -3309,7 +3421,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3449,7 +3563,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3465,7 +3579,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: An unread notification 'Event rescheduled' is listed with the message '"SPM53 Harbour Confirmed Gala" has a new date and time: 25 Apr 2028, 09:00–12:00.' and the event 'SPM53 Harbour Confirmed Gala' with its reference.
+Step 4: Anita Devi's list has no notification about 'SPM53 Harbour Confirmed Gala'.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -3475,7 +3594,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3604,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -3493,7 +3616,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -3501,7 +3628,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3641,7 +3770,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3657,7 +3786,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 3: A green alert 'You're registered for this event.' appears, with the status badge 'Registered'.
+Step 4: An unread notification 'Registration confirmed' is listed with the message 'You're registered for "SPM53 Harbour Postponed Fair".' and the event 'SPM53 Harbour Postponed Fair' with its reference.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -3667,7 +3801,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -3677,7 +3811,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -3685,7 +3823,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -3693,7 +3835,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3839,7 +3983,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -3855,7 +3999,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 4: The message 'The event is confirmed. The organiser can now see the arrangements.' is shown and the status badge changes to 'Confirmed'.
+Step 7: The status badge changes to 'Completed'.
+Step 9: Two new unread notifications are listed, newest first: 'Event completed' ('"SPM53 Harbour Finished Dinner" has been marked completed.') and 'Event confirmed' ('"SPM53 Harbour Ready Launch" is confirmed.').</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -3863,7 +4013,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -3871,7 +4025,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -3879,7 +4037,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -3887,7 +4049,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46325</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -3895,7 +4059,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>a22feeb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4026,7 +4194,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4036,13 +4204,19 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12" ht="12.5" customHeight="1">
+    <row r="12" ht="75" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Step 2: The event's page opens with the status badge 'Submitted'.
+Step 4: An unread notification 'New event request submitted' is listed with the message '"SPM53 Harbour Draft Summit" has been submitted and needs a coordinator assigned.' and the event 'SPM53 Harbour Draft Summit' with its reference.
+Step 6: Grace Lim's list has the same unread notification.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -4062,7 +4236,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -4070,7 +4248,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -4078,7 +4260,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="12" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -4232,7 +4416,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4248,7 +4432,15 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 5: The status badge changes to 'Postponed'.
+Step 9: The status badge changes to 'Cancelled'.
+Step 11: Two new unread notifications are listed, newest first: 'Event cancelled' ('"SPM53 Harbour Cancelled Summit" has been cancelled.', with no reason) and 'Event postponed' ('"SPM53 Harbour Postponed Fair" has been postponed. Reason: The keynote speaker is unwell.').
+Step 13: Lee Wei Ming's list has the same two unread notifications, above 'Registration confirmed'.
+Step 15: Anita Devi's list has no notification about 'SPM53 Harbour Postponed Fair' or 'SPM53 Harbour Cancelled Summit'.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -4256,7 +4448,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -4264,7 +4460,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -4272,7 +4472,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -4280,7 +4484,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46325</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -4288,7 +4494,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>a22feeb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4419,7 +4629,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4435,7 +4645,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: Rachel Ng's Notifications page opens. Note the number on the bell at the top of the page (no number when nothing is unread).
+Step 6: A green 'Request approved' alert is shown.
+Step 7: 'Event request approved' ('"SPM53 Harbour Live Update" has been approved.') is at the top of the list, marked 'Unread', dated just now. The bell shows one more than in Step 1.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -4445,7 +4661,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -4455,7 +4671,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -4463,7 +4683,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -4471,7 +4695,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -4608,7 +4834,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4624,7 +4850,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 1: The event page for 'SPM53 Harbour Live Update' opens on its Overview, with the status badge 'Approved'.
+Step 2: The 'Event request approved' notification is no longer marked 'Unread'.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -4634,7 +4865,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4875,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -4652,7 +4887,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -4660,7 +4899,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -4724,7 +4965,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="44.5" customHeight="1">
+    <row r="4" ht="75" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -4737,7 +4978,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44.5" customHeight="1">
+    <row r="5" ht="112.5" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -4755,7 +4996,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="17.5" customHeight="1">
+    <row r="6" ht="25" customHeight="1">
       <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -4768,7 +5009,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
+    <row r="7" ht="87.5" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -4803,7 +5044,7 @@
         <v>46325</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -4819,7 +5060,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 5: A green alert 'Anita Devi has been added to the registration list.' is shown, and Anita Devi is listed as Registered with 'Added by Daniel Tan'.
+Step 7: An unread notification 'Registration confirmed' is listed with the message 'You're registered for "SPM53 Harbour Confirmed Gala".' and the event 'SPM53 Harbour Confirmed Gala' with its reference.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -4827,7 +5073,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -4835,7 +5085,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -4843,7 +5097,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -4851,7 +5109,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46325</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -4859,7 +5119,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>a22feeb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4988,7 +5252,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5004,7 +5268,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 3: 'SPM53 Harbour Draft Summit' leaves the 'Awaiting assignment' list.
+Step 5: An unread notification 'Coordinator assigned' is listed with the message 'Daniel Tan is now the coordinator for "SPM53 Harbour Draft Summit".' and the event 'SPM53 Harbour Draft Summit' with its reference.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -5012,7 +5281,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -5020,7 +5293,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -5028,7 +5305,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -5036,7 +5317,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46325</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -5044,7 +5327,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>a22feeb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5168,7 +5455,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5184,7 +5471,11 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 2: An unread notification 'You have been assigned an event' is listed with the message 'You are now the coordinator for "SPM53 Harbour Draft Summit".'</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -5192,7 +5483,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -5200,7 +5495,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -5208,7 +5507,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -5216,7 +5519,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46325</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -5224,7 +5529,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>a22feeb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5363,7 +5672,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5379,7 +5688,14 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 6: The message '"SPM53 Harbour Draft Summit" has been reassigned from Daniel Tan to Priya Raj.' appears.
+Step 8: An unread notification 'You have been assigned an event' is listed with the message 'You are now the coordinator for "SPM53 Harbour Draft Summit".'
+Step 10: An unread notification 'An event has been reassigned' is listed with the message '"SPM53 Harbour Draft Summit" has been reassigned to Priya Raj. You are no longer its coordinator.'
+Step 12: A new unread 'Coordinator assigned' notification reads 'Priya Raj is now the coordinator for "SPM53 Harbour Draft Summit".', above the one naming Daniel Tan from SPM-53-TC02.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -5389,7 +5705,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -5399,7 +5715,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -5407,7 +5727,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -5415,7 +5739,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -5558,7 +5884,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5574,7 +5900,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 5: The clarification request is sent and the event stays Under review.
+Step 7: An unread notification 'Clarification requested' is listed with the message 'Your coordinator asked for clarification on "SPM53 Harbour Clarity Forum": Can the forum start at 10:00 instead of 09:00?' and the event 'SPM53 Harbour Clarity Forum' with its reference.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -5584,7 +5915,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -5594,7 +5925,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -5602,7 +5937,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -5610,7 +5949,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -5752,7 +6093,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5768,7 +6109,12 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 4: The event page opens with a green message 'Your updated request has been sent to Daniel Tan. It stays Under review.'
+Step 6: An unread notification 'Clarification answered' is listed with the message 'The organiser has responded to your clarification request on "SPM53 Harbour Clarity Forum".'</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -5778,7 +6124,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -5788,7 +6134,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -5796,7 +6146,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -5804,7 +6158,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -5954,7 +6310,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -5970,7 +6326,14 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 4: A green 'Request approved' alert is shown and the status badge changes to 'Approved'.
+Step 8: A green 'Request rejected' alert is shown and the status badge changes to 'Rejected'.
+Step 10: Two new unread notifications are listed, newest first: 'Event request rejected' ('"SPM53 Harbour Rejected Brief" has been rejected. Reason: The brief duplicates the March town hall; please merge the two.') and 'Event request approved' ('"SPM53 Harbour Clarity Forum" has been approved.').
+Step 12: Grace Lim's list has no 'Event request approved' or 'Event request rejected' notification for either event.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -5978,7 +6341,11 @@
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -5986,7 +6353,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -5994,7 +6365,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -6002,7 +6377,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46325</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
@@ -6010,7 +6387,11 @@
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>a22feeb</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6146,7 +6527,7 @@
         <v>46324</v>
       </c>
     </row>
-    <row r="10"/>
+    <row r="10" ht="12.5" customHeight="1"/>
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -6162,7 +6543,13 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Step 6: 'Booking request sent to Venue Staff.' is shown.
+Step 8: An unread notification 'Venue booking request to review' is listed with the message '"SPM53 Harbour Booking Review" requests SPM53 Hall (SPM53-HAL) on 23 Mar 2028, 09:00–12:00.' and the event 'SPM53 Harbour Booking Review' with its reference.
+Step 10: Marcus Wong's list has the same unread notification.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
@@ -6172,7 +6559,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -6182,7 +6569,11 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
@@ -6190,7 +6581,11 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi Chua</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
@@ -6198,7 +6593,9 @@
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="17" t="n">
+        <v>46324</v>
+      </c>
     </row>
     <row r="17" ht="12.5" customHeight="1">
       <c r="A17" s="3" t="inlineStr">

</xml_diff>